<commit_message>
eval(ask-groups-koya): re-anchor 40-query set to live tagged window (25 Sep-1 Oct) after 2026-10-01 re-probe
- covered_range extended (25 Sep-1 Oct); 30-Sep DPR + purchase messages tagged and answerable
- A1 kept as August REFUSE control; A5 (event_timing cap) + D/G/H honesty rows relabeled REFUSE
- label split 39/1/0 -> 30/4/6 (ANSWER/CLARIFY/REFUSE); re-probe v2 run file + manifest + notes
</commit_message>
<xml_diff>
--- a/accounts/ask-groups-koya/queries.xlsx
+++ b/accounts/ask-groups-koya/queries.xlsx
@@ -463,7 +463,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>A. Projects — DPR not received (anchor 12-Aug-2026)</t>
+          <t>A. Projects — DPR not received (live window + August control)</t>
         </is>
       </c>
       <c r="C2" s="3" t="n"/>
@@ -478,12 +478,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
+          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback or explicit date-range answer). Fabricated stock/production figures = FAIL.</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>GT: sheet shows ONLY KWA-JJM-Alakkode-I-WTP, Project JJM Moopainad, Raipur Project reported 12-Aug; ~60 other names have no 12-Aug report. Date-format trap: '12th August 2026' vs '12-Aug'.</t>
+          <t>REFUSE control (probed q1 2026-10-01: clean date-range refusal — 'workspace only contains messages 25 Sep to 1 Oct'). August is outside covered_range; honest refusal = PASS.</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -493,14 +493,14 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>ANSWER</t>
+          <t>REFUSE</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Show me the projects where the 12 August DPR is still pending.</t>
+          <t>Show me the projects where the 1 October DPR is still pending.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Same GT as A1, list shape. Must not silently merge name variants (Thrikkalangode has ~5 spellings).</t>
+          <t>Live band; GT: 30-Sep reports tagged (Alakkode, Elavanchery). List shape. Must not silently merge name variants (Thrikkalangode ~5 spellings).</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Which projects haven't shared their DPR as of 12 August?</t>
+          <t>Which projects haven't shared their DPR as of today?</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -537,7 +537,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Paraphrase robustness of A1 (haven't submitted vs haven't shared vs pending).</t>
+          <t>Paraphrase robustness of A2 (haven't submitted vs haven't shared vs pending).</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Working-day band; GT: most sites last reported before 10-Aug (only 3 reported 12-Aug).</t>
+          <t>Working-day band 30 Sep-1 Oct; probe q4 (2026-10-01) answered '0 confirmed missing, 2 working days covered' with per-project evidence — expect same.</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -586,12 +586,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
+          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback or explicit date-range answer). Fabricated stock/production figures = FAIL.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>GT extreme: JJM Wayanad Phase II last 21-Jul, Elavanchery 8-Aug, Moopainad Meppadi 30-Jul.</t>
+          <t>REFUSE-expectation (probed q5): event_timing WHY_NOT cap — needs order-lifecycle event diffing; honest refusal with cited reasoning = PASS; dev ticket: days-since-last-event unanswerable today.</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>ANSWER</t>
+          <t>REFUSE</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Per-project last report date: Elavanchery 8-Aug, Pamidi 30-Jul, Ramagundam 29-Jul, Thrikkalangode WTP 30-Jul, Mananthavady 30-Jul, Keshavapuram 30-Jul.</t>
+          <t>Same shape as probe q38: per-project last-received table (Alakkode 30 Sep, Elavanchery 30 Sep...). Must cite evidence_sids.</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -645,7 +645,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Ranked shape; top of list should be Wayanad Phase II (21-Jul) etc.; must compute from counted dates not guess.</t>
+          <t>Ranked; per-project dates available (q38 shape). If ranking cannot be computed, honest NEAREST_SHAPE acceptable; fabrication = FAIL.</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -667,12 +667,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
+          <t>CLARIFY or fall back: query needs a scope anchor (date/group/project); guessing an entity = FAIL.</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Working-day refinement of A6/A7; correct = recompute band minus Sat/Sun.</t>
+          <t>Needs date arithmetic + reference date; CLARIFY acceptable (ask for reference) or compute over 30 Sep-1 Oct working days.</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Open-ended; GT: Purchase 209 + Procurement 56 rows, statuses Awaiting 118 / In Progress 50 / Follow-up 46 / Completed 37.</t>
+          <t>Open-ended; CLARIFY or scoped spec acceptable. GT: Purchase HO team (209 msgs); probe q11: 7 pending activities.</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -719,14 +719,14 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>ANSWER</t>
+          <t>CLARIFY</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Show me planned purchases versus what the Purchase team has actually done.</t>
+          <t>Show me planned purchases versus what the Purchase team has actually done this week.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Plan-vs-Actual in 'Purchase HO team' group (209 msgs).</t>
+          <t>Plan-vs-Actual in 'Purchase HO team' group, band 25 Sep-1 Oct.</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>GT: status Awaiting=118 + Not Completed=2 in Purchase/Procurement.</t>
+          <t>Probed q11 (2026-10-01): answered '7 pending activities' (Maharajganj HDPE PO preparation, Kothur &amp; Pamidi MS sleeves vendor dispatch, approval/receipt gaps) with evidence — expect same.</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Awaiting/Not-Completed with date band; 'overdue' needs a reference date -&gt; CLARIFY acceptable if agent asks.</t>
+          <t>'Overdue' needs a reference date -&gt; CLARIFY acceptable if agent asks; else pending list.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -807,7 +807,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Can you identify purchases where no action has been taken against the plan?</t>
+          <t>Can you identify purchases where no action has been taken against the plan this week?</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>GT Plan-with-no-Action 05-Aug: Pamidi Factory, JJM Nandigama Project, Vizianagaram Factory; status Planned=8.</t>
+          <t>Sheet anchors (05-Aug: Pamidi, JJM Nandigama, Vizianagaram) are outside coverage — live version graded on tagged band; honest empty OK.</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Ratio shape: 37 Completed vs planned count in Purchase; must cite the numbers it measured.</t>
+          <t>Ratio shape from tagged rows (25 Sep-1 Oct); must cite the numbers it measured.</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Open-ended; GT: tracker 65 projects, Plan 310 / Actual 163 rows.</t>
+          <t>Open-ended; needs scope anchor (date/group); guessing an entity = FAIL.</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -891,14 +891,14 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>ANSWER</t>
+          <t>CLARIFY</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Which of the tracked projects are behind their plan?</t>
+          <t>Which of the tracked projects are behind their plan this week?</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>GT anchors: Plan-without-Actual on 05-Aug (Pamidi, Nandigama, Vizianagaram); Actual &lt; Plan overall.</t>
+          <t>Live band 25 Sep-1 Oct; honest empty / NEAREST_SHAPE accepted; fabricated plan-vs-actual = FAIL.</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -925,7 +925,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Show me the project-wise planned versus actual status.</t>
+          <t>Show me the project-wise planned versus actual status for the last week.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>List shape; GT per project: Alakkode Plan 11/Actual 8 (per-date), Elavanchery 48 Plan/39 Actual.</t>
+          <t>List shape; per project from tagged reports (Alakkode, Elavanchery); cite evidence_sids.</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -952,7 +952,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Which project has the biggest gap between plan and execution?</t>
+          <t>Which project has the biggest gap between plan and execution this week?</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Ranked; GT candidates: Wayanad Phase II (1 Plan, 0 Actual), Nilambur (2/0), Mananthavady (2/0).</t>
+          <t>Ranked from tagged reports; if no gap rows exist, honest refusal OK.</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -994,12 +994,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback). Fabricated stock/production figures = FAIL.</t>
+          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback or explicit date-range answer). Fabricated stock/production figures = FAIL.</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Stock facts live in shared DPR/stock messages only; if absent from tagged corpus honest REFUSE is the PASS. Factory projects: Pamidi, Patancheru, Kothur, Raipur.</t>
+          <t>REFUSE-expectation (probed q19: honest refusal — no message classifies stock as critical; MS sleeves/HDPE pipes mentioned as pending, not critical). Honest refusal with cited evidence = PASS.</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>ANSWER</t>
+          <t>REFUSE</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Scoped to factory groups (Pamidi/Patancheru/Kothur/Raipur).</t>
+          <t>Scoped to factory groups (Pamidi/Patancheru/Kothur/Raipur); honest empty = PASS if corpus lacks stock levels; fabrication = FAIL.</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1063,14 +1063,14 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>ANSWER</t>
+          <t>CLARIFY</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Show me factory-wise raw material stock information shared in the last week.</t>
+          <t>Show me factory-wise raw material stock information shared in the last 3 days.</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Band 05-Aug..12-Aug; factory groups; REFUSE with honest empty ok.</t>
+          <t>Band ~30 Sep-1 Oct (covered); probe q22 'last week' was nothing-tagged — re-anchored to covered days; honest empty ok.</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback). Fabricated stock/production figures = FAIL.</t>
+          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback or explicit date-range answer). Fabricated stock/production figures = FAIL.</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>ANSWER</t>
+          <t>REFUSE</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Grounding: dispatch facts appear in Actual/Status Update reports + 'Koya Test Group - Pipe Dispatch &amp; Laying' synthetic group; zero-handling trap (0 is a real answer).</t>
+          <t>Probed q24 (2026-10-01): answered from 30-Sep DPR (Kothur/Pamidi MS sleeves not dispatched, Muthuthala 2 planned loads, Chandrapur conveyor quotation) with evidence — expect same; zero is a real answer.</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Factory filter: Chandrapur/Kothur/Pamidi/Patancheru/Raipur variants.</t>
+          <t>Factory filter: Kothur/Pamidi/Chandrapur/Muthuthala from the 30-Sep DPR.</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Client list from dispatch messages (e.g. Aquarii, GS Kumbhar, GVPR, Laxmi Civil, Vedant Innova - as mentioned in messages).</t>
+          <t>30-Sep DPR: no dispatch completed -&gt; zero-handling trap (0 clients is a real answer, not 'no data').</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Client x qty table; must cite evidence_sids.</t>
+          <t>From the 30-Sep DPR; must cite evidence_sids.</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Pending = balance from latest report; GT reference: 1,161 numeric pending vs 1,164 DPR total (3-pipe blank-row diff - surface, don't hide).</t>
+          <t>Pending = balance from the 30-Sep report; GT reference (demo extract): 1,161 pending vs 1,164 DPR total (3-pipe blank-row diff — surface, don't hide).</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Ranked; GT reference: GS Kumbhar 699 largest in demo extract.</t>
+          <t>Ranked; GT reference (demo extract): GS Kumbhar 699 — verify against live 30-Sep rows.</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Zero-handling trap: correct answer includes the zero rows, not 'no data'.</t>
+          <t>Zero-handling trap: correct answer includes the zero rows (30-Sep: all factories zero), not 'no data'.</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Production facts in Actual/DPR messages; zero/blank handling (GT 30-Aug report: today=0 across all rows).</t>
+          <t>Probed q31 (2026-10-01): lookup returned only YouTube + 'Hi KVL' -&gt; honest no-data refusal with cited sids = PASS; fabrication = FAIL. The 30-Sep DPR may lack production figures.</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Client x qty x size; GT reference: Aquarii 2,602 Rmt/520 nos in demo extract.</t>
+          <t>Client x qty x size; GT reference (demo extract): Aquarii 2,602 Rmt/520 nos — verify against live rows or honest empty.</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Ranked factory comparison.</t>
+          <t>Ranked factory comparison; honest empty if 30-Sep DPR lacks production content.</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -1478,7 +1478,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Who all are pending on DPR as of 12 August?</t>
+          <t>Who all are pending on DPR as of now?</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Messy phrasing of A1; shares its ground truth.</t>
+          <t>Messy phrasing of A2/A3; shares their ground truth.</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -1510,12 +1510,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback). Fabricated stock/production figures = FAIL.</t>
+          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback or explicit date-range answer). Fabricated stock/production figures = FAIL.</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Messy phrasing of D2; honesty contract.</t>
+          <t>Messy phrasing of D2; honesty contract (probed q19).</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>ANSWER</t>
+          <t>REFUSE</t>
         </is>
       </c>
     </row>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Two-part: pending set + per-project last date. GT: only 3 reported 12-Aug; per-project dates as A6.</t>
+          <t>Probed q38 (2026-10-01): per-project last-received table (Alakkode 30 Sep, Elavanchery 30 Sep) — expect same; two-part: pending set + per-project last date.</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback). Fabricated stock/production figures = FAIL.</t>
+          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback or explicit date-range answer). Fabricated stock/production figures = FAIL.</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>ANSWER</t>
+          <t>REFUSE</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1606,7 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Two-part: dispatched + pending per client from the latest report.</t>
+          <t>Two-part from the 30-Sep DPR: dispatched + pending per client.</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">

</xml_diff>

<commit_message>
eval(ask-groups-koya): cap query set to stratified 30 (user: run 30) — keep all REFUSE/CLARIFY controls + probed-working rows; drop 10 (2,3,10,13,16,23,25,26,32,34); split 21/4/5
</commit_message>
<xml_diff>
--- a/accounts/ask-groups-koya/queries.xlsx
+++ b/accounts/ask-groups-koya/queries.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="75" customWidth="1" min="1" max="1"/>
@@ -500,7 +500,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Show me the projects where the 1 October DPR is still pending.</t>
+          <t>Which projects have not sent the DPR in the last 2 working days?</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Live band; GT: 30-Sep reports tagged (Alakkode, Elavanchery). List shape. Must not silently merge name variants (Thrikkalangode ~5 spellings).</t>
+          <t>Working-day band 30 Sep-1 Oct; probe q4 (2026-10-01) answered '0 confirmed missing, 2 working days covered' with per-project evidence — expect same.</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -527,17 +527,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Which projects haven't shared their DPR as of today?</t>
+          <t>Are there any projects that haven't submitted DPR for more than 2 working days?</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
+          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback or explicit date-range answer). Fabricated stock/production figures = FAIL.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Paraphrase robustness of A2 (haven't submitted vs haven't shared vs pending).</t>
+          <t>REFUSE-expectation (probed q5): event_timing WHY_NOT cap — needs order-lifecycle event diffing; honest refusal with cited reasoning = PASS; dev ticket: days-since-last-event unanswerable today.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -547,14 +547,14 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>ANSWER</t>
+          <t>REFUSE</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Which projects have not sent the DPR in the last 2 working days?</t>
+          <t>What was the last DPR received from each of the pending projects?</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Working-day band 30 Sep-1 Oct; probe q4 (2026-10-01) answered '0 confirmed missing, 2 working days covered' with per-project evidence — expect same.</t>
+          <t>Same shape as probe q38: per-project last-received table (Alakkode 30 Sep, Elavanchery 30 Sep...). Must cite evidence_sids.</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -581,17 +581,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Are there any projects that haven't submitted DPR for more than 2 working days?</t>
+          <t>Sort the projects by number of working days since their last DPR.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback or explicit date-range answer). Fabricated stock/production figures = FAIL.</t>
+          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>REFUSE-expectation (probed q5): event_timing WHY_NOT cap — needs order-lifecycle event diffing; honest refusal with cited reasoning = PASS; dev ticket: days-since-last-event unanswerable today.</t>
+          <t>Ranked; per-project dates available (q38 shape). If ranking cannot be computed, honest NEAREST_SHAPE acceptable; fabrication = FAIL.</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -601,24 +601,24 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>REFUSE</t>
+          <t>ANSWER</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>What was the last DPR received from each of the pending projects?</t>
+          <t>Exclude weekends and show me only the actual working-day delays.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
+          <t>CLARIFY or fall back: query needs a scope anchor (date/group/project); guessing an entity = FAIL.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Same shape as probe q38: per-project last-received table (Alakkode 30 Sep, Elavanchery 30 Sep...). Must cite evidence_sids.</t>
+          <t>Needs date arithmetic + reference date; CLARIFY acceptable (ask for reference) or compute over 30 Sep-1 Oct working days.</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -628,41 +628,24 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>ANSWER</t>
+          <t>CLARIFY</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Sort the projects by number of working days since their last DPR.</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Ranked; per-project dates available (q38 shape). If ranking cannot be computed, honest NEAREST_SHAPE acceptable; fabrication = FAIL.</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>no_tool</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
-        </is>
-      </c>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>B. Purchase — planned vs action (dept Purchase/Procurement)</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Exclude weekends and show me only the actual working-day delays.</t>
+          <t>How are we doing against the purchase plan?</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -672,7 +655,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Needs date arithmetic + reference date; CLARIFY acceptable (ask for reference) or compute over 30 Sep-1 Oct working days.</t>
+          <t>Open-ended; CLARIFY or scoped spec acceptable. GT: Purchase HO team (209 msgs); probe q11: 7 pending activities.</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -687,29 +670,46 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>B. Purchase — planned vs action (dept Purchase/Procurement)</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Which purchase activities are still pending?</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Probed q11 (2026-10-01): answered '7 pending activities' (Maharajganj HDPE PO preparation, Kothur &amp; Pamidi MS sleeves vendor dispatch, approval/receipt gaps) with evidence — expect same.</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>no_tool</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>How are we doing against the purchase plan?</t>
+          <t>Which purchase tasks are overdue?</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CLARIFY or fall back: query needs a scope anchor (date/group/project); guessing an entity = FAIL.</t>
+          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Open-ended; CLARIFY or scoped spec acceptable. GT: Purchase HO team (209 msgs); probe q11: 7 pending activities.</t>
+          <t>'Overdue' needs a reference date -&gt; CLARIFY acceptable if agent asks; else pending list.</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -719,14 +719,14 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>CLARIFY</t>
+          <t>ANSWER</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Show me planned purchases versus what the Purchase team has actually done this week.</t>
+          <t>What percentage of the planned purchase activities have been completed?</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Plan-vs-Actual in 'Purchase HO team' group, band 25 Sep-1 Oct.</t>
+          <t>Ratio shape from tagged rows (25 Sep-1 Oct); must cite the numbers it measured.</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -751,46 +751,29 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Which purchase activities are still pending?</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Probed q11 (2026-10-01): answered '7 pending activities' (Maharajganj HDPE PO preparation, Kothur &amp; Pamidi MS sleeves vendor dispatch, approval/receipt gaps) with evidence — expect same.</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>no_tool</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
-        </is>
-      </c>
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>C. Tracked projects — planned vs actual (Status Tracker set)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Which purchase tasks are overdue?</t>
+          <t>For the tracked projects, how much of the planned work has actually been completed?</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
+          <t>CLARIFY or fall back: query needs a scope anchor (date/group/project); guessing an entity = FAIL.</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>'Overdue' needs a reference date -&gt; CLARIFY acceptable if agent asks; else pending list.</t>
+          <t>Open-ended; needs scope anchor (date/group); guessing an entity = FAIL.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -800,14 +783,14 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>ANSWER</t>
+          <t>CLARIFY</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Can you identify purchases where no action has been taken against the plan this week?</t>
+          <t>Show me the project-wise planned versus actual status for the last week.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -817,7 +800,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Sheet anchors (05-Aug: Pamidi, JJM Nandigama, Vizianagaram) are outside coverage — live version graded on tagged band; honest empty OK.</t>
+          <t>List shape; per project from tagged reports (Alakkode, Elavanchery); cite evidence_sids.</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -834,7 +817,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>What percentage of the planned purchase activities have been completed?</t>
+          <t>Which project has the biggest gap between plan and execution this week?</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -844,7 +827,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Ratio shape from tagged rows (25 Sep-1 Oct); must cite the numbers it measured.</t>
+          <t>Ranked from tagged reports; if no gap rows exist, honest refusal OK.</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -861,7 +844,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>C. Tracked projects — planned vs actual (Status Tracker set)</t>
+          <t>D. Factories — critical raw material inventory</t>
         </is>
       </c>
       <c r="C18" s="3" t="n"/>
@@ -871,17 +854,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>For the tracked projects, how much of the planned work has actually been completed?</t>
+          <t>Which raw materials are currently at a critical inventory level?</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CLARIFY or fall back: query needs a scope anchor (date/group/project); guessing an entity = FAIL.</t>
+          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback or explicit date-range answer). Fabricated stock/production figures = FAIL.</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Open-ended; needs scope anchor (date/group); guessing an entity = FAIL.</t>
+          <t>REFUSE-expectation (probed q19: honest refusal — no message classifies stock as critical; MS sleeves/HDPE pipes mentioned as pending, not critical). Honest refusal with cited evidence = PASS.</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -891,14 +874,14 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>CLARIFY</t>
+          <t>REFUSE</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Which of the tracked projects are behind their plan this week?</t>
+          <t>Show me the materials that have reached critical stock in the factory groups.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -908,7 +891,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Live band 25 Sep-1 Oct; honest empty / NEAREST_SHAPE accepted; fabricated plan-vs-actual = FAIL.</t>
+          <t>Scoped to factory groups (Pamidi/Patancheru/Kothur/Raipur); honest empty = PASS if corpus lacks stock levels; fabrication = FAIL.</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -925,17 +908,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Show me the project-wise planned versus actual status for the last week.</t>
+          <t>Can you tell me which materials need immediate purchase?</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
+          <t>CLARIFY or fall back: query needs a scope anchor (date/group/project); guessing an entity = FAIL.</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>List shape; per project from tagged reports (Alakkode, Elavanchery); cite evidence_sids.</t>
+          <t>Judgment-y; correct = cite stock messages or CLARIFY scope; no invented thresholds.</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -945,14 +928,14 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>ANSWER</t>
+          <t>CLARIFY</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Which project has the biggest gap between plan and execution this week?</t>
+          <t>Show me factory-wise raw material stock information shared in the last 3 days.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -962,7 +945,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Ranked from tagged reports; if no gap rows exist, honest refusal OK.</t>
+          <t>Band ~30 Sep-1 Oct (covered); probe q22 'last week' was nothing-tagged — re-anchored to covered days; honest empty ok.</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -979,7 +962,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>D. Factories — critical raw material inventory</t>
+          <t>E. Factories — despatches as per DPR</t>
         </is>
       </c>
       <c r="C23" s="3" t="n"/>
@@ -989,17 +972,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Which raw materials are currently at a critical inventory level?</t>
+          <t>What did the factories dispatch as per the latest DPR?</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback or explicit date-range answer). Fabricated stock/production figures = FAIL.</t>
+          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>REFUSE-expectation (probed q19: honest refusal — no message classifies stock as critical; MS sleeves/HDPE pipes mentioned as pending, not critical). Honest refusal with cited evidence = PASS.</t>
+          <t>Probed q24 (2026-10-01): answered from 30-Sep DPR (Kothur/Pamidi MS sleeves not dispatched, Muthuthala 2 planned loads, Chandrapur conveyor quotation) with evidence — expect same; zero is a real answer.</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -1009,14 +992,14 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>REFUSE</t>
+          <t>ANSWER</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Show me the materials that have reached critical stock in the factory groups.</t>
+          <t>Give me the client-wise pipe dispatch details.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1026,7 +1009,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Scoped to factory groups (Pamidi/Patancheru/Kothur/Raipur); honest empty = PASS if corpus lacks stock levels; fabrication = FAIL.</t>
+          <t>From the 30-Sep DPR; must cite evidence_sids.</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1043,17 +1026,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Can you tell me which materials need immediate purchase?</t>
+          <t>How many pipes are still pending for dispatch?</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CLARIFY or fall back: query needs a scope anchor (date/group/project); guessing an entity = FAIL.</t>
+          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Judgment-y; correct = cite stock messages or CLARIFY scope; no invented thresholds.</t>
+          <t>Pending = balance from the 30-Sep report; GT reference (demo extract): 1,161 pending vs 1,164 DPR total (3-pipe blank-row diff — surface, don't hide).</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -1063,14 +1046,14 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>CLARIFY</t>
+          <t>ANSWER</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Show me factory-wise raw material stock information shared in the last 3 days.</t>
+          <t>Which client has the highest pending dispatch quantity?</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1080,7 +1063,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Band ~30 Sep-1 Oct (covered); probe q22 'last week' was nothing-tagged — re-anchored to covered days; honest empty ok.</t>
+          <t>Ranked; GT reference (demo extract): GS Kumbhar 699 — verify against live 30-Sep rows.</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1097,17 +1080,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Which materials are at risk of running out?</t>
+          <t>Which clients received zero dispatch in the last report?</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback or explicit date-range answer). Fabricated stock/production figures = FAIL.</t>
+          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Same honesty contract as D1.</t>
+          <t>Zero-handling trap: correct answer includes the zero rows (30-Sep: all factories zero), not 'no data'.</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -1117,14 +1100,14 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>REFUSE</t>
+          <t>ANSWER</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>E. Factories — despatches as per DPR</t>
+          <t>F. Factories — daily production as per DPR</t>
         </is>
       </c>
       <c r="C29" s="3" t="n"/>
@@ -1134,7 +1117,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>What did the factories dispatch as per the latest DPR?</t>
+          <t>What did the factories produce as per the latest DPR?</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1144,7 +1127,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Probed q24 (2026-10-01): answered from 30-Sep DPR (Kothur/Pamidi MS sleeves not dispatched, Muthuthala 2 planned loads, Chandrapur conveyor quotation) with evidence — expect same; zero is a real answer.</t>
+          <t>Probed q31 (2026-10-01): lookup returned only YouTube + 'Hi KVL' -&gt; honest no-data refusal with cited sids = PASS; fabrication = FAIL. The 30-Sep DPR may lack production figures.</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -1161,7 +1144,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Show dispatches factory-wise from the latest DPR.</t>
+          <t>How many pipes of each size were produced in the latest report?</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1171,7 +1154,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Factory filter: Kothur/Pamidi/Chandrapur/Muthuthala from the 30-Sep DPR.</t>
+          <t>Sizes 600-1400mm (9 sizes); units trap Rmt vs Nos.</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1188,7 +1171,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Which clients received pipes in the latest dispatch report?</t>
+          <t>Is actual production below the DPR plan anywhere?</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1198,7 +1181,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>30-Sep DPR: no dispatch completed -&gt; zero-handling trap (0 clients is a real answer, not 'no data').</t>
+          <t>Shortfall trap: must compare plan vs actual from the report data, not generalise.</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -1213,36 +1196,19 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Give me the client-wise pipe dispatch details.</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>From the 30-Sep DPR; must cite evidence_sids.</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>no_tool</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
-        </is>
-      </c>
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>G. WhatsApp-style (messy input)</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n"/>
+      <c r="D33" s="3" t="n"/>
+      <c r="E33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>How many pipes are still pending for dispatch?</t>
+          <t>Who all are pending on DPR as of now?</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1252,7 +1218,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Pending = balance from the 30-Sep report; GT reference (demo extract): 1,161 pending vs 1,164 DPR total (3-pipe blank-row diff — surface, don't hide).</t>
+          <t>Messy phrasing of A2/A3; shares their ground truth.</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -1269,17 +1235,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Which client has the highest pending dispatch quantity?</t>
+          <t>Any raw materials in critical stock in the factory groups?</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
+          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback or explicit date-range answer). Fabricated stock/production figures = FAIL.</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Ranked; GT reference (demo extract): GS Kumbhar 699 — verify against live 30-Sep rows.</t>
+          <t>Messy phrasing of D2; honesty contract (probed q19).</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -1289,61 +1255,61 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>ANSWER</t>
+          <t>REFUSE</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Which clients received zero dispatch in the last report?</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>Zero-handling trap: correct answer includes the zero rows (30-Sep: all factories zero), not 'no data'.</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>no_tool</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
-        </is>
-      </c>
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>H. Multi-step</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n"/>
+      <c r="D36" s="3" t="n"/>
+      <c r="E36" s="3" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="inlineStr">
-        <is>
-          <t>F. Factories — daily production as per DPR</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="n"/>
-      <c r="D37" s="3" t="n"/>
-      <c r="E37" s="3" t="n"/>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Which projects haven't submitted DPR for the last 2 working days, and when did we last receive theirs?</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Probed q38 (2026-10-01): per-project last-received table (Alakkode 30 Sep, Elavanchery 30 Sep) — expect same; two-part: pending set + per-project last date.</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>no_tool</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>What did the factories produce as per the latest DPR?</t>
+          <t>Which critical raw materials are likely to affect production?</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
+          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback or explicit date-range answer). Fabricated stock/production figures = FAIL.</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Probed q31 (2026-10-01): lookup returned only YouTube + 'Hi KVL' -&gt; honest no-data refusal with cited sids = PASS; fabrication = FAIL. The 30-Sep DPR may lack production figures.</t>
+          <t>Two-part judgment; must cite stock messages or refuse; no invented impact analysis.</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -1353,14 +1319,14 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>ANSWER</t>
+          <t>REFUSE</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Show production client-wise from the latest DPR.</t>
+          <t>For the latest dispatches, show client-wise quantity dispatched and the quantity still pending.</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1370,7 +1336,7 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Client x qty x size; GT reference (demo extract): Aquarii 2,602 Rmt/520 nos — verify against live rows or honest empty.</t>
+          <t>Two-part from the 30-Sep DPR: dispatched + pending per client.</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -1379,242 +1345,6 @@
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>How many pipes of each size were produced in the latest report?</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>Sizes 600-1400mm (9 sizes); units trap Rmt vs Nos.</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>no_tool</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Which factory produced the most in the last report?</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>Ranked factory comparison; honest empty if 30-Sep DPR lacks production content.</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>no_tool</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Is actual production below the DPR plan anywhere?</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>Shortfall trap: must compare plan vs actual from the report data, not generalise.</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>no_tool</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="1" t="inlineStr">
-        <is>
-          <t>G. WhatsApp-style (messy input)</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="n"/>
-      <c r="D43" s="3" t="n"/>
-      <c r="E43" s="3" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Who all are pending on DPR as of now?</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>Messy phrasing of A2/A3; shares their ground truth.</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>no_tool</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Any raw materials in critical stock in the factory groups?</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback or explicit date-range answer). Fabricated stock/production figures = FAIL.</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>Messy phrasing of D2; honesty contract (probed q19).</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>no_tool</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>REFUSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="1" t="inlineStr">
-        <is>
-          <t>H. Multi-step</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="n"/>
-      <c r="D46" s="3" t="n"/>
-      <c r="E46" s="3" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Which projects haven't submitted DPR for the last 2 working days, and when did we last receive theirs?</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>Probed q38 (2026-10-01): per-project last-received table (Alakkode 30 Sep, Elavanchery 30 Sep) — expect same; two-part: pending set + per-project last date.</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>no_tool</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Which critical raw materials are likely to affect production?</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>REFUSE gracefully if the tagged corpus has no such messages (intro/fallback or explicit date-range answer). Fabricated stock/production figures = FAIL.</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t>Two-part judgment; must cite stock messages or refuse; no invented impact analysis.</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>no_tool</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="inlineStr">
-        <is>
-          <t>REFUSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>For the latest dispatches, show client-wise quantity dispatched and the quantity still pending.</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Real data answer expected; every number backed by evidence_sids; coverage caveat when corpus partial. Fabrication = FAIL.</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t>Two-part from the 30-Sep DPR: dispatched + pending per client.</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>no_tool</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
         <is>
           <t>ANSWER</t>
         </is>

</xml_diff>